<commit_message>
Update reference nutrition data files
Adds tenpercent.xlsx and refreshes MegaCoffee/TheVenti reference data
in raw/DB (source material for future admin data entry, not yet
imported into the app).
</commit_message>
<xml_diff>
--- a/raw/DB/MegaCoffee.xlsx
+++ b/raw/DB/MegaCoffee.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Desktop\기타서류\3.홈페이지 아이디어\DB\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/6f05ca6d36262a21/Desktop/caffeinenote/raw/DB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{10ACBECA-3972-413D-8B98-BF66FA8A4D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="2" documentId="8_{10ACBECA-3972-413D-8B98-BF66FA8A4D97}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF35B6C6-C356-4151-8B39-4A37EADD9FEB}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="13965" windowHeight="14460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2205" yWindow="2205" windowWidth="16200" windowHeight="9307" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="메가커피" sheetId="1" r:id="rId1"/>
@@ -2565,7 +2565,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F160"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="20" customWidth="1"/>
@@ -5786,9 +5786,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.73046875" defaultRowHeight="14.25"/>
   <cols>
-    <col min="1" max="1" width="70" customWidth="1"/>
+    <col min="1" max="1" width="108.46484375" customWidth="1"/>
     <col min="2" max="2" width="30" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>